<commit_message>
Credit link points to GitHub
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Grade-6_Annual-Plan_2026-2027_English/Grade-6_English_Annual-Plan_2026-2027.xlsx
+++ b/Grade-6_Annual-Plan_2026-2027_English/Grade-6_English_Annual-Plan_2026-2027.xlsx
@@ -1726,7 +1726,7 @@
     <row r="47" ht="14" customHeight="1">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>Prepared by Ogün Aydın · CC BY 4.0: free to use, share and adapt with credit · codeberg.org/helinesca/ingilizce-6-materyaller</t>
+          <t>Prepared by Ogün Aydın · CC BY 4.0: free to use, share and adapt with credit · github.com/ogunaydin89/ingilizce-6-materyaller</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1782,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;7 Prepared by Ogün Aydın · CC BY 4.0: free to use, share and adapt with credit · codeberg.org/helinesca/ingilizce-6-materyaller</oddFooter>
+    <oddFooter>&amp;C&amp;7 Prepared by Ogün Aydın · CC BY 4.0: free to use, share and adapt with credit · github.com/ogunaydin89/ingilizce-6-materyaller</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>